<commit_message>
update type input field
</commit_message>
<xml_diff>
--- a/cypress/fixtures/run-log.xlsx
+++ b/cypress/fixtures/run-log.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AD6"/>
+  <dimension ref="A1:AD32"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str" xml:space="preserve">
@@ -888,9 +888,2011 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>(243)</v>
+      </c>
+      <c r="B7" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C7" t="str">
+        <v>73399</v>
+      </c>
+      <c r="D7" t="str">
+        <v>388673145</v>
+      </c>
+      <c r="E7" t="str">
+        <v>NGUYỄN VĂN DƯỜNG</v>
+      </c>
+      <c r="F7" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M7" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N7" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O7" t="str">
+        <v>0</v>
+      </c>
+      <c r="P7" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>0</v>
+      </c>
+      <c r="R7" t="str">
+        <v>0</v>
+      </c>
+      <c r="S7" t="str">
+        <v>0</v>
+      </c>
+      <c r="T7" t="str">
+        <v>0</v>
+      </c>
+      <c r="U7" t="str">
+        <v>4</v>
+      </c>
+      <c r="V7" t="str">
+        <v>0</v>
+      </c>
+      <c r="W7" t="str">
+        <v>3</v>
+      </c>
+      <c r="X7" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y7" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z7" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB7" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD7" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>(245)</v>
+      </c>
+      <c r="B8" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C8" t="str">
+        <v>73401</v>
+      </c>
+      <c r="D8" t="str">
+        <v>359757527</v>
+      </c>
+      <c r="E8" t="str">
+        <v>NGUYỄN THANH NHÀN</v>
+      </c>
+      <c r="F8" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M8" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N8" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O8" t="str">
+        <v>1</v>
+      </c>
+      <c r="P8" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>0</v>
+      </c>
+      <c r="R8" t="str">
+        <v>0</v>
+      </c>
+      <c r="S8" t="str">
+        <v>0</v>
+      </c>
+      <c r="T8" t="str">
+        <v>0</v>
+      </c>
+      <c r="U8" t="str">
+        <v>4</v>
+      </c>
+      <c r="V8" t="str">
+        <v>0</v>
+      </c>
+      <c r="W8" t="str">
+        <v>3</v>
+      </c>
+      <c r="X8" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y8" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z8" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD8" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>(246)</v>
+      </c>
+      <c r="B9" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C9" t="str">
+        <v>73402</v>
+      </c>
+      <c r="D9" t="str">
+        <v>382211425</v>
+      </c>
+      <c r="E9" t="str">
+        <v>HUỲNH HOÀNG DŨNG</v>
+      </c>
+      <c r="F9" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J9" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M9" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N9" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O9" t="str">
+        <v>1</v>
+      </c>
+      <c r="P9" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>0</v>
+      </c>
+      <c r="R9" t="str">
+        <v>0</v>
+      </c>
+      <c r="S9" t="str">
+        <v>0</v>
+      </c>
+      <c r="T9" t="str">
+        <v>0</v>
+      </c>
+      <c r="U9" t="str">
+        <v>3</v>
+      </c>
+      <c r="V9" t="str">
+        <v>0</v>
+      </c>
+      <c r="W9" t="str">
+        <v>2</v>
+      </c>
+      <c r="X9" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y9" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z9" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB9" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD9" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>(247)</v>
+      </c>
+      <c r="B10" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C10" t="str">
+        <v>73403</v>
+      </c>
+      <c r="D10" t="str">
+        <v>913613458</v>
+      </c>
+      <c r="E10" t="str">
+        <v>ĐINH THÀNH NGUYÊN</v>
+      </c>
+      <c r="F10" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L10" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M10" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N10" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O10" t="str">
+        <v>0</v>
+      </c>
+      <c r="P10" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>0</v>
+      </c>
+      <c r="R10" t="str">
+        <v>0</v>
+      </c>
+      <c r="S10" t="str">
+        <v>0</v>
+      </c>
+      <c r="T10" t="str">
+        <v>0</v>
+      </c>
+      <c r="U10" t="str">
+        <v>2</v>
+      </c>
+      <c r="V10" t="str">
+        <v>0</v>
+      </c>
+      <c r="W10" t="str">
+        <v>1</v>
+      </c>
+      <c r="X10" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y10" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z10" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB10" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD10" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>(249)</v>
+      </c>
+      <c r="B11" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C11" t="str">
+        <v>73405</v>
+      </c>
+      <c r="D11" t="str">
+        <v>834994432</v>
+      </c>
+      <c r="E11" t="str">
+        <v>NGUYỄN VĂN NHÁNH</v>
+      </c>
+      <c r="F11" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J11" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L11" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M11" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N11" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O11" t="str">
+        <v>0</v>
+      </c>
+      <c r="P11" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>0</v>
+      </c>
+      <c r="R11" t="str">
+        <v>0</v>
+      </c>
+      <c r="S11" t="str">
+        <v>0</v>
+      </c>
+      <c r="T11" t="str">
+        <v>0</v>
+      </c>
+      <c r="U11" t="str">
+        <v>4</v>
+      </c>
+      <c r="V11" t="str">
+        <v>0</v>
+      </c>
+      <c r="W11" t="str">
+        <v>3</v>
+      </c>
+      <c r="X11" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y11" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z11" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB11" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD11" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>(250)</v>
+      </c>
+      <c r="B12" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C12" t="str">
+        <v>73406</v>
+      </c>
+      <c r="D12" t="str">
+        <v>936735077</v>
+      </c>
+      <c r="E12" t="str">
+        <v>NGUYỄN MINH TRƯỜNG</v>
+      </c>
+      <c r="F12" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J12" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L12" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M12" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N12" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O12" t="str">
+        <v>1</v>
+      </c>
+      <c r="P12" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>0</v>
+      </c>
+      <c r="R12" t="str">
+        <v>0</v>
+      </c>
+      <c r="S12" t="str">
+        <v>0</v>
+      </c>
+      <c r="T12" t="str">
+        <v>0</v>
+      </c>
+      <c r="U12" t="str">
+        <v>3</v>
+      </c>
+      <c r="V12" t="str">
+        <v>0</v>
+      </c>
+      <c r="W12" t="str">
+        <v>2</v>
+      </c>
+      <c r="X12" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y12" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z12" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB12" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD12" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>(251)</v>
+      </c>
+      <c r="B13" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C13" t="str">
+        <v>73407</v>
+      </c>
+      <c r="D13" t="str">
+        <v>356309142</v>
+      </c>
+      <c r="E13" t="str">
+        <v>TRẦN VĂN VĨNH</v>
+      </c>
+      <c r="F13" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J13" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L13" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M13" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N13" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O13" t="str">
+        <v>0</v>
+      </c>
+      <c r="P13" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>0</v>
+      </c>
+      <c r="R13" t="str">
+        <v>0</v>
+      </c>
+      <c r="S13" t="str">
+        <v>0</v>
+      </c>
+      <c r="T13" t="str">
+        <v>0</v>
+      </c>
+      <c r="U13" t="str">
+        <v>2</v>
+      </c>
+      <c r="V13" t="str">
+        <v>0</v>
+      </c>
+      <c r="W13" t="str">
+        <v>1</v>
+      </c>
+      <c r="X13" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y13" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z13" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB13" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD13" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>(256)</v>
+      </c>
+      <c r="B14" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C14" t="str">
+        <v>73412</v>
+      </c>
+      <c r="D14" t="str">
+        <v>388443780</v>
+      </c>
+      <c r="E14" t="str">
+        <v>PHAN VĂN BE</v>
+      </c>
+      <c r="F14" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J14" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L14" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M14" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N14" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O14" t="str">
+        <v>0</v>
+      </c>
+      <c r="P14" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>0</v>
+      </c>
+      <c r="R14" t="str">
+        <v>0</v>
+      </c>
+      <c r="S14" t="str">
+        <v>0</v>
+      </c>
+      <c r="T14" t="str">
+        <v>0</v>
+      </c>
+      <c r="U14" t="str">
+        <v>4</v>
+      </c>
+      <c r="V14" t="str">
+        <v>0</v>
+      </c>
+      <c r="W14" t="str">
+        <v>3</v>
+      </c>
+      <c r="X14" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y14" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z14" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB14" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD14" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>(243)</v>
+      </c>
+      <c r="B15" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C15" t="str">
+        <v>73399</v>
+      </c>
+      <c r="D15" t="str">
+        <v>388673145</v>
+      </c>
+      <c r="E15" t="str">
+        <v>NGUYỄN VĂN DƯỜNG</v>
+      </c>
+      <c r="F15" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J15" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L15" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M15" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N15" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O15" t="str">
+        <v>0</v>
+      </c>
+      <c r="P15" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>0</v>
+      </c>
+      <c r="R15" t="str">
+        <v>0</v>
+      </c>
+      <c r="S15" t="str">
+        <v>0</v>
+      </c>
+      <c r="T15" t="str">
+        <v>0</v>
+      </c>
+      <c r="U15" t="str">
+        <v>4</v>
+      </c>
+      <c r="V15" t="str">
+        <v>0</v>
+      </c>
+      <c r="W15" t="str">
+        <v>3</v>
+      </c>
+      <c r="X15" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y15" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z15" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB15" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD15" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>(245)</v>
+      </c>
+      <c r="B16" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C16" t="str">
+        <v>73401</v>
+      </c>
+      <c r="D16" t="str">
+        <v>359757527</v>
+      </c>
+      <c r="E16" t="str">
+        <v>NGUYỄN THANH NHÀN</v>
+      </c>
+      <c r="F16" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J16" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K16" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L16" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M16" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N16" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O16" t="str">
+        <v>1</v>
+      </c>
+      <c r="P16" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>0</v>
+      </c>
+      <c r="R16" t="str">
+        <v>0</v>
+      </c>
+      <c r="S16" t="str">
+        <v>0</v>
+      </c>
+      <c r="T16" t="str">
+        <v>0</v>
+      </c>
+      <c r="U16" t="str">
+        <v>4</v>
+      </c>
+      <c r="V16" t="str">
+        <v>0</v>
+      </c>
+      <c r="W16" t="str">
+        <v>3</v>
+      </c>
+      <c r="X16" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y16" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z16" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB16" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD16" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>(246)</v>
+      </c>
+      <c r="B17" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C17" t="str">
+        <v>73402</v>
+      </c>
+      <c r="D17" t="str">
+        <v>382211425</v>
+      </c>
+      <c r="E17" t="str">
+        <v>HUỲNH HOÀNG DŨNG</v>
+      </c>
+      <c r="F17" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J17" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L17" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M17" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N17" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O17" t="str">
+        <v>1</v>
+      </c>
+      <c r="P17" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>0</v>
+      </c>
+      <c r="R17" t="str">
+        <v>0</v>
+      </c>
+      <c r="S17" t="str">
+        <v>0</v>
+      </c>
+      <c r="T17" t="str">
+        <v>0</v>
+      </c>
+      <c r="U17" t="str">
+        <v>3</v>
+      </c>
+      <c r="V17" t="str">
+        <v>0</v>
+      </c>
+      <c r="W17" t="str">
+        <v>2</v>
+      </c>
+      <c r="X17" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y17" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z17" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB17" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD17" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>(247)</v>
+      </c>
+      <c r="B18" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C18" t="str">
+        <v>73403</v>
+      </c>
+      <c r="D18" t="str">
+        <v>913613458</v>
+      </c>
+      <c r="E18" t="str">
+        <v>ĐINH THÀNH NGUYÊN</v>
+      </c>
+      <c r="F18" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J18" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L18" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M18" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N18" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O18" t="str">
+        <v>0</v>
+      </c>
+      <c r="P18" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>0</v>
+      </c>
+      <c r="R18" t="str">
+        <v>0</v>
+      </c>
+      <c r="S18" t="str">
+        <v>0</v>
+      </c>
+      <c r="T18" t="str">
+        <v>0</v>
+      </c>
+      <c r="U18" t="str">
+        <v>2</v>
+      </c>
+      <c r="V18" t="str">
+        <v>0</v>
+      </c>
+      <c r="W18" t="str">
+        <v>1</v>
+      </c>
+      <c r="X18" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y18" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z18" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB18" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD18" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>(249)</v>
+      </c>
+      <c r="B19" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C19" t="str">
+        <v>73405</v>
+      </c>
+      <c r="D19" t="str">
+        <v>834994432</v>
+      </c>
+      <c r="E19" t="str">
+        <v>NGUYỄN VĂN NHÁNH</v>
+      </c>
+      <c r="F19" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J19" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L19" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M19" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N19" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O19" t="str">
+        <v>0</v>
+      </c>
+      <c r="P19" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>0</v>
+      </c>
+      <c r="R19" t="str">
+        <v>0</v>
+      </c>
+      <c r="S19" t="str">
+        <v>0</v>
+      </c>
+      <c r="T19" t="str">
+        <v>0</v>
+      </c>
+      <c r="U19" t="str">
+        <v>4</v>
+      </c>
+      <c r="V19" t="str">
+        <v>0</v>
+      </c>
+      <c r="W19" t="str">
+        <v>3</v>
+      </c>
+      <c r="X19" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y19" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z19" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB19" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD19" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>(250)</v>
+      </c>
+      <c r="B20" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C20" t="str">
+        <v>73406</v>
+      </c>
+      <c r="D20" t="str">
+        <v>936735077</v>
+      </c>
+      <c r="E20" t="str">
+        <v>NGUYỄN MINH TRƯỜNG</v>
+      </c>
+      <c r="F20" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J20" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K20" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L20" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M20" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N20" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O20" t="str">
+        <v>1</v>
+      </c>
+      <c r="P20" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>0</v>
+      </c>
+      <c r="R20" t="str">
+        <v>0</v>
+      </c>
+      <c r="S20" t="str">
+        <v>0</v>
+      </c>
+      <c r="T20" t="str">
+        <v>0</v>
+      </c>
+      <c r="U20" t="str">
+        <v>3</v>
+      </c>
+      <c r="V20" t="str">
+        <v>0</v>
+      </c>
+      <c r="W20" t="str">
+        <v>2</v>
+      </c>
+      <c r="X20" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y20" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z20" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB20" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD20" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>(251)</v>
+      </c>
+      <c r="B21" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C21" t="str">
+        <v>73407</v>
+      </c>
+      <c r="D21" t="str">
+        <v>356309142</v>
+      </c>
+      <c r="E21" t="str">
+        <v>TRẦN VĂN VĨNH</v>
+      </c>
+      <c r="F21" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J21" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K21" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L21" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M21" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N21" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O21" t="str">
+        <v>0</v>
+      </c>
+      <c r="P21" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>0</v>
+      </c>
+      <c r="R21" t="str">
+        <v>0</v>
+      </c>
+      <c r="S21" t="str">
+        <v>0</v>
+      </c>
+      <c r="T21" t="str">
+        <v>0</v>
+      </c>
+      <c r="U21" t="str">
+        <v>2</v>
+      </c>
+      <c r="V21" t="str">
+        <v>0</v>
+      </c>
+      <c r="W21" t="str">
+        <v>1</v>
+      </c>
+      <c r="X21" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y21" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z21" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB21" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD21" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>(256)</v>
+      </c>
+      <c r="B22" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C22" t="str">
+        <v>73412</v>
+      </c>
+      <c r="D22" t="str">
+        <v>388443780</v>
+      </c>
+      <c r="E22" t="str">
+        <v>PHAN VĂN BE</v>
+      </c>
+      <c r="F22" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J22" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L22" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M22" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N22" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O22" t="str">
+        <v>0</v>
+      </c>
+      <c r="P22" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>0</v>
+      </c>
+      <c r="R22" t="str">
+        <v>0</v>
+      </c>
+      <c r="S22" t="str">
+        <v>0</v>
+      </c>
+      <c r="T22" t="str">
+        <v>0</v>
+      </c>
+      <c r="U22" t="str">
+        <v>4</v>
+      </c>
+      <c r="V22" t="str">
+        <v>0</v>
+      </c>
+      <c r="W22" t="str">
+        <v>3</v>
+      </c>
+      <c r="X22" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y22" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z22" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB22" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD22" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>(243)</v>
+      </c>
+      <c r="B23" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C23" t="str">
+        <v>73399</v>
+      </c>
+      <c r="D23" t="str">
+        <v>388673145</v>
+      </c>
+      <c r="E23" t="str">
+        <v>NGUYỄN VĂN DƯỜNG</v>
+      </c>
+      <c r="F23" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J23" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L23" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M23" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N23" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O23" t="str">
+        <v>0</v>
+      </c>
+      <c r="P23" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>0</v>
+      </c>
+      <c r="R23" t="str">
+        <v>0</v>
+      </c>
+      <c r="S23" t="str">
+        <v>0</v>
+      </c>
+      <c r="T23" t="str">
+        <v>0</v>
+      </c>
+      <c r="U23" t="str">
+        <v>4</v>
+      </c>
+      <c r="V23" t="str">
+        <v>0</v>
+      </c>
+      <c r="W23" t="str">
+        <v>3</v>
+      </c>
+      <c r="X23" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y23" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z23" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB23" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD23" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>(245)</v>
+      </c>
+      <c r="B24" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C24" t="str">
+        <v>73401</v>
+      </c>
+      <c r="D24" t="str">
+        <v>359757527</v>
+      </c>
+      <c r="E24" t="str">
+        <v>NGUYỄN THANH NHÀN</v>
+      </c>
+      <c r="F24" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J24" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L24" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M24" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N24" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O24" t="str">
+        <v>1</v>
+      </c>
+      <c r="P24" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>0</v>
+      </c>
+      <c r="R24" t="str">
+        <v>0</v>
+      </c>
+      <c r="S24" t="str">
+        <v>0</v>
+      </c>
+      <c r="T24" t="str">
+        <v>0</v>
+      </c>
+      <c r="U24" t="str">
+        <v>4</v>
+      </c>
+      <c r="V24" t="str">
+        <v>0</v>
+      </c>
+      <c r="W24" t="str">
+        <v>3</v>
+      </c>
+      <c r="X24" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y24" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z24" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB24" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD24" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>(246)</v>
+      </c>
+      <c r="B25" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C25" t="str">
+        <v>73402</v>
+      </c>
+      <c r="D25" t="str">
+        <v>382211425</v>
+      </c>
+      <c r="E25" t="str">
+        <v>HUỲNH HOÀNG DŨNG</v>
+      </c>
+      <c r="F25" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J25" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K25" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L25" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M25" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N25" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O25" t="str">
+        <v>1</v>
+      </c>
+      <c r="P25" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>0</v>
+      </c>
+      <c r="R25" t="str">
+        <v>0</v>
+      </c>
+      <c r="S25" t="str">
+        <v>0</v>
+      </c>
+      <c r="T25" t="str">
+        <v>0</v>
+      </c>
+      <c r="U25" t="str">
+        <v>3</v>
+      </c>
+      <c r="V25" t="str">
+        <v>0</v>
+      </c>
+      <c r="W25" t="str">
+        <v>2</v>
+      </c>
+      <c r="X25" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y25" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z25" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB25" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD25" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>(247)</v>
+      </c>
+      <c r="B26" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C26" t="str">
+        <v>73403</v>
+      </c>
+      <c r="D26" t="str">
+        <v>913613458</v>
+      </c>
+      <c r="E26" t="str">
+        <v>ĐINH THÀNH NGUYÊN</v>
+      </c>
+      <c r="F26" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L26" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M26" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N26" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O26" t="str">
+        <v>0</v>
+      </c>
+      <c r="P26" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>0</v>
+      </c>
+      <c r="R26" t="str">
+        <v>0</v>
+      </c>
+      <c r="S26" t="str">
+        <v>0</v>
+      </c>
+      <c r="T26" t="str">
+        <v>0</v>
+      </c>
+      <c r="U26" t="str">
+        <v>2</v>
+      </c>
+      <c r="V26" t="str">
+        <v>0</v>
+      </c>
+      <c r="W26" t="str">
+        <v>1</v>
+      </c>
+      <c r="X26" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y26" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z26" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB26" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD26" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>(249)</v>
+      </c>
+      <c r="B27" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C27" t="str">
+        <v>73405</v>
+      </c>
+      <c r="D27" t="str">
+        <v>834994432</v>
+      </c>
+      <c r="E27" t="str">
+        <v>NGUYỄN VĂN NHÁNH</v>
+      </c>
+      <c r="F27" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K27" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L27" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M27" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N27" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O27" t="str">
+        <v>0</v>
+      </c>
+      <c r="P27" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>0</v>
+      </c>
+      <c r="R27" t="str">
+        <v>0</v>
+      </c>
+      <c r="S27" t="str">
+        <v>0</v>
+      </c>
+      <c r="T27" t="str">
+        <v>0</v>
+      </c>
+      <c r="U27" t="str">
+        <v>4</v>
+      </c>
+      <c r="V27" t="str">
+        <v>0</v>
+      </c>
+      <c r="W27" t="str">
+        <v>3</v>
+      </c>
+      <c r="X27" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y27" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z27" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB27" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD27" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>(250)</v>
+      </c>
+      <c r="B28" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C28" t="str">
+        <v>73406</v>
+      </c>
+      <c r="D28" t="str">
+        <v>936735077</v>
+      </c>
+      <c r="E28" t="str">
+        <v>NGUYỄN MINH TRƯỜNG</v>
+      </c>
+      <c r="F28" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L28" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M28" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N28" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O28" t="str">
+        <v>1</v>
+      </c>
+      <c r="P28" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>0</v>
+      </c>
+      <c r="R28" t="str">
+        <v>0</v>
+      </c>
+      <c r="S28" t="str">
+        <v>0</v>
+      </c>
+      <c r="T28" t="str">
+        <v>0</v>
+      </c>
+      <c r="U28" t="str">
+        <v>3</v>
+      </c>
+      <c r="V28" t="str">
+        <v>0</v>
+      </c>
+      <c r="W28" t="str">
+        <v>2</v>
+      </c>
+      <c r="X28" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y28" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z28" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB28" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD28" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>(251)</v>
+      </c>
+      <c r="B29" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C29" t="str">
+        <v>73407</v>
+      </c>
+      <c r="D29" t="str">
+        <v>356309142</v>
+      </c>
+      <c r="E29" t="str">
+        <v>TRẦN VĂN VĨNH</v>
+      </c>
+      <c r="F29" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L29" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M29" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N29" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O29" t="str">
+        <v>0</v>
+      </c>
+      <c r="P29" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>0</v>
+      </c>
+      <c r="R29" t="str">
+        <v>0</v>
+      </c>
+      <c r="S29" t="str">
+        <v>0</v>
+      </c>
+      <c r="T29" t="str">
+        <v>0</v>
+      </c>
+      <c r="U29" t="str">
+        <v>2</v>
+      </c>
+      <c r="V29" t="str">
+        <v>0</v>
+      </c>
+      <c r="W29" t="str">
+        <v>1</v>
+      </c>
+      <c r="X29" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y29" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z29" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB29" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD29" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>(256)</v>
+      </c>
+      <c r="B30" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C30" t="str">
+        <v>73412</v>
+      </c>
+      <c r="D30" t="str">
+        <v>388443780</v>
+      </c>
+      <c r="E30" t="str">
+        <v>PHAN VĂN BE</v>
+      </c>
+      <c r="F30" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L30" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M30" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N30" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O30" t="str">
+        <v>0</v>
+      </c>
+      <c r="P30" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>0</v>
+      </c>
+      <c r="R30" t="str">
+        <v>0</v>
+      </c>
+      <c r="S30" t="str">
+        <v>0</v>
+      </c>
+      <c r="T30" t="str">
+        <v>0</v>
+      </c>
+      <c r="U30" t="str">
+        <v>4</v>
+      </c>
+      <c r="V30" t="str">
+        <v>0</v>
+      </c>
+      <c r="W30" t="str">
+        <v>3</v>
+      </c>
+      <c r="X30" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y30" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z30" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB30" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD30" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>(243)</v>
+      </c>
+      <c r="B31" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C31" t="str">
+        <v>73399</v>
+      </c>
+      <c r="D31" t="str">
+        <v>388673145</v>
+      </c>
+      <c r="E31" t="str">
+        <v>NGUYỄN VĂN DƯỜNG</v>
+      </c>
+      <c r="F31" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L31" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M31" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N31" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O31" t="str">
+        <v>0</v>
+      </c>
+      <c r="P31" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>0</v>
+      </c>
+      <c r="R31" t="str">
+        <v>0</v>
+      </c>
+      <c r="S31" t="str">
+        <v>0</v>
+      </c>
+      <c r="T31" t="str">
+        <v>0</v>
+      </c>
+      <c r="U31" t="str">
+        <v>4</v>
+      </c>
+      <c r="V31" t="str">
+        <v>0</v>
+      </c>
+      <c r="W31" t="str">
+        <v>3</v>
+      </c>
+      <c r="X31" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y31" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z31" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB31" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD31" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>(245)</v>
+      </c>
+      <c r="B32" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-THT HKD Thanh Mai</v>
+      </c>
+      <c r="C32" t="str">
+        <v>73401</v>
+      </c>
+      <c r="D32" t="str">
+        <v>359757527</v>
+      </c>
+      <c r="E32" t="str">
+        <v>NGUYỄN THANH NHÀN</v>
+      </c>
+      <c r="F32" t="str">
+        <v>HỘ KINH DOANH THANH MAI</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L32" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M32" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N32" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O32" t="str">
+        <v>1</v>
+      </c>
+      <c r="P32" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>0</v>
+      </c>
+      <c r="R32" t="str">
+        <v>0</v>
+      </c>
+      <c r="S32" t="str">
+        <v>0</v>
+      </c>
+      <c r="T32" t="str">
+        <v>0</v>
+      </c>
+      <c r="U32" t="str">
+        <v>4</v>
+      </c>
+      <c r="V32" t="str">
+        <v>0</v>
+      </c>
+      <c r="W32" t="str">
+        <v>3</v>
+      </c>
+      <c r="X32" t="str">
+        <v>4/6/26</v>
+      </c>
+      <c r="Y32" t="str">
+        <v>7/10/26</v>
+      </c>
+      <c r="Z32" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB32" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD32" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AD6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AD32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix bug: skip disable intended practice
</commit_message>
<xml_diff>
--- a/cypress/fixtures/run-log.xlsx
+++ b/cypress/fixtures/run-log.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE177"/>
+  <dimension ref="A1:AE193"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str" xml:space="preserve">
@@ -14863,9 +14863,1337 @@
         <v/>
       </c>
     </row>
+    <row r="178" xml:space="preserve">
+      <c r="A178" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B178" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C178" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D178" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E178" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F178" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J178" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K178" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L178" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M178" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N178" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O178" t="str">
+        <v>1</v>
+      </c>
+      <c r="P178" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q178" t="str">
+        <v>0</v>
+      </c>
+      <c r="R178" t="str">
+        <v>0</v>
+      </c>
+      <c r="S178" t="str">
+        <v>0</v>
+      </c>
+      <c r="T178" t="str">
+        <v>0</v>
+      </c>
+      <c r="U178" t="str">
+        <v>4</v>
+      </c>
+      <c r="V178" t="str">
+        <v>0</v>
+      </c>
+      <c r="W178" t="str">
+        <v>2</v>
+      </c>
+      <c r="X178" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y178" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z178" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB178" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD178" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE178" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="179" xml:space="preserve">
+      <c r="A179" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B179" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C179" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D179" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E179" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F179" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J179" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K179" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L179" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M179" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N179" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O179" t="str">
+        <v>1</v>
+      </c>
+      <c r="P179" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q179" t="str">
+        <v>0</v>
+      </c>
+      <c r="R179" t="str">
+        <v>0</v>
+      </c>
+      <c r="S179" t="str">
+        <v>0</v>
+      </c>
+      <c r="T179" t="str">
+        <v>0</v>
+      </c>
+      <c r="U179" t="str">
+        <v>4</v>
+      </c>
+      <c r="V179" t="str">
+        <v>0</v>
+      </c>
+      <c r="W179" t="str">
+        <v>2</v>
+      </c>
+      <c r="X179" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y179" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z179" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB179" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD179" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE179" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="180" xml:space="preserve">
+      <c r="A180" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B180" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C180" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D180" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E180" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F180" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J180" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K180" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L180" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M180" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N180" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O180" t="str">
+        <v>1</v>
+      </c>
+      <c r="P180" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q180" t="str">
+        <v>0</v>
+      </c>
+      <c r="R180" t="str">
+        <v>0</v>
+      </c>
+      <c r="S180" t="str">
+        <v>0</v>
+      </c>
+      <c r="T180" t="str">
+        <v>0</v>
+      </c>
+      <c r="U180" t="str">
+        <v>4</v>
+      </c>
+      <c r="V180" t="str">
+        <v>0</v>
+      </c>
+      <c r="W180" t="str">
+        <v>2</v>
+      </c>
+      <c r="X180" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y180" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z180" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB180" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD180" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE180" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="181" xml:space="preserve">
+      <c r="A181" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B181" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C181" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D181" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E181" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F181" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J181" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K181" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L181" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M181" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N181" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O181" t="str">
+        <v>1</v>
+      </c>
+      <c r="P181" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q181" t="str">
+        <v>0</v>
+      </c>
+      <c r="R181" t="str">
+        <v>0</v>
+      </c>
+      <c r="S181" t="str">
+        <v>0</v>
+      </c>
+      <c r="T181" t="str">
+        <v>0</v>
+      </c>
+      <c r="U181" t="str">
+        <v>4</v>
+      </c>
+      <c r="V181" t="str">
+        <v>0</v>
+      </c>
+      <c r="W181" t="str">
+        <v>2</v>
+      </c>
+      <c r="X181" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y181" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z181" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB181" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD181" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE181" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="182" xml:space="preserve">
+      <c r="A182" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B182" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C182" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D182" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E182" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F182" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J182" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K182" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L182" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M182" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N182" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O182" t="str">
+        <v>1</v>
+      </c>
+      <c r="P182" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q182" t="str">
+        <v>0</v>
+      </c>
+      <c r="R182" t="str">
+        <v>0</v>
+      </c>
+      <c r="S182" t="str">
+        <v>0</v>
+      </c>
+      <c r="T182" t="str">
+        <v>0</v>
+      </c>
+      <c r="U182" t="str">
+        <v>4</v>
+      </c>
+      <c r="V182" t="str">
+        <v>0</v>
+      </c>
+      <c r="W182" t="str">
+        <v>2</v>
+      </c>
+      <c r="X182" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y182" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z182" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB182" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD182" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE182" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="183" xml:space="preserve">
+      <c r="A183" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B183" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C183" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D183" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E183" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F183" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J183" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K183" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L183" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M183" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N183" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O183" t="str">
+        <v>1</v>
+      </c>
+      <c r="P183" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q183" t="str">
+        <v>0</v>
+      </c>
+      <c r="R183" t="str">
+        <v>0</v>
+      </c>
+      <c r="S183" t="str">
+        <v>0</v>
+      </c>
+      <c r="T183" t="str">
+        <v>0</v>
+      </c>
+      <c r="U183" t="str">
+        <v>4</v>
+      </c>
+      <c r="V183" t="str">
+        <v>0</v>
+      </c>
+      <c r="W183" t="str">
+        <v>2</v>
+      </c>
+      <c r="X183" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y183" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z183" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB183" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD183" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE183" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="184" xml:space="preserve">
+      <c r="A184" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B184" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C184" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D184" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E184" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F184" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J184" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K184" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L184" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M184" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N184" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O184" t="str">
+        <v>1</v>
+      </c>
+      <c r="P184" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q184" t="str">
+        <v>0</v>
+      </c>
+      <c r="R184" t="str">
+        <v>0</v>
+      </c>
+      <c r="S184" t="str">
+        <v>0</v>
+      </c>
+      <c r="T184" t="str">
+        <v>0</v>
+      </c>
+      <c r="U184" t="str">
+        <v>4</v>
+      </c>
+      <c r="V184" t="str">
+        <v>0</v>
+      </c>
+      <c r="W184" t="str">
+        <v>2</v>
+      </c>
+      <c r="X184" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y184" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z184" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB184" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD184" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE184" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="185" xml:space="preserve">
+      <c r="A185" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B185" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C185" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D185" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E185" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F185" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J185" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K185" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L185" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M185" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N185" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O185" t="str">
+        <v>1</v>
+      </c>
+      <c r="P185" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q185" t="str">
+        <v>0</v>
+      </c>
+      <c r="R185" t="str">
+        <v>0</v>
+      </c>
+      <c r="S185" t="str">
+        <v>0</v>
+      </c>
+      <c r="T185" t="str">
+        <v>0</v>
+      </c>
+      <c r="U185" t="str">
+        <v>4</v>
+      </c>
+      <c r="V185" t="str">
+        <v>0</v>
+      </c>
+      <c r="W185" t="str">
+        <v>2</v>
+      </c>
+      <c r="X185" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y185" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z185" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB185" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD185" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE185" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="186" xml:space="preserve">
+      <c r="A186" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B186" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C186" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D186" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E186" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F186" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J186" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K186" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L186" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M186" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N186" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O186" t="str">
+        <v>1</v>
+      </c>
+      <c r="P186" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q186" t="str">
+        <v>0</v>
+      </c>
+      <c r="R186" t="str">
+        <v>0</v>
+      </c>
+      <c r="S186" t="str">
+        <v>0</v>
+      </c>
+      <c r="T186" t="str">
+        <v>0</v>
+      </c>
+      <c r="U186" t="str">
+        <v>4</v>
+      </c>
+      <c r="V186" t="str">
+        <v>0</v>
+      </c>
+      <c r="W186" t="str">
+        <v>2</v>
+      </c>
+      <c r="X186" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y186" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z186" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB186" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD186" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE186" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="187" xml:space="preserve">
+      <c r="A187" t="str">
+        <v>(1252)</v>
+      </c>
+      <c r="B187" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group - HTX An Hoà</v>
+      </c>
+      <c r="C187" t="str">
+        <v>74110</v>
+      </c>
+      <c r="D187" t="str">
+        <v>946756347</v>
+      </c>
+      <c r="E187" t="str">
+        <v>TRẦN VĂN KHÁNH</v>
+      </c>
+      <c r="F187" t="str">
+        <v>HỢP TÁC XÃ NÔNG NGHIỆP AN HÒA</v>
+      </c>
+      <c r="J187" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K187" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L187" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M187" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N187" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O187" t="str">
+        <v>0</v>
+      </c>
+      <c r="P187" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q187" t="str">
+        <v>0</v>
+      </c>
+      <c r="R187" t="str">
+        <v>0</v>
+      </c>
+      <c r="S187" t="str">
+        <v>0</v>
+      </c>
+      <c r="T187" t="str">
+        <v>0</v>
+      </c>
+      <c r="U187" t="str">
+        <v>2</v>
+      </c>
+      <c r="V187" t="str">
+        <v>0</v>
+      </c>
+      <c r="W187" t="str">
+        <v>1</v>
+      </c>
+      <c r="X187" t="str">
+        <v>5/17/26</v>
+      </c>
+      <c r="Y187" t="str">
+        <v>8/20/26</v>
+      </c>
+      <c r="Z187" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB187" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD187" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE187" t="str">
+        <v>Skipped: Intended practices disabled (program stage)</v>
+      </c>
+    </row>
+    <row r="188" xml:space="preserve">
+      <c r="A188" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B188" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C188" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D188" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E188" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F188" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J188" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K188" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L188" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M188" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N188" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O188" t="str">
+        <v>1</v>
+      </c>
+      <c r="P188" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q188" t="str">
+        <v>0</v>
+      </c>
+      <c r="R188" t="str">
+        <v>0</v>
+      </c>
+      <c r="S188" t="str">
+        <v>0</v>
+      </c>
+      <c r="T188" t="str">
+        <v>0</v>
+      </c>
+      <c r="U188" t="str">
+        <v>4</v>
+      </c>
+      <c r="V188" t="str">
+        <v>0</v>
+      </c>
+      <c r="W188" t="str">
+        <v>2</v>
+      </c>
+      <c r="X188" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y188" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z188" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB188" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD188" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE188" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="189" xml:space="preserve">
+      <c r="A189" t="str">
+        <v>(1252)</v>
+      </c>
+      <c r="B189" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group - HTX An Hoà</v>
+      </c>
+      <c r="C189" t="str">
+        <v>74110</v>
+      </c>
+      <c r="D189" t="str">
+        <v>946756347</v>
+      </c>
+      <c r="E189" t="str">
+        <v>TRẦN VĂN KHÁNH</v>
+      </c>
+      <c r="F189" t="str">
+        <v>HỢP TÁC XÃ NÔNG NGHIỆP AN HÒA</v>
+      </c>
+      <c r="J189" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K189" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L189" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M189" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N189" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O189" t="str">
+        <v>0</v>
+      </c>
+      <c r="P189" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q189" t="str">
+        <v>0</v>
+      </c>
+      <c r="R189" t="str">
+        <v>0</v>
+      </c>
+      <c r="S189" t="str">
+        <v>0</v>
+      </c>
+      <c r="T189" t="str">
+        <v>0</v>
+      </c>
+      <c r="U189" t="str">
+        <v>2</v>
+      </c>
+      <c r="V189" t="str">
+        <v>0</v>
+      </c>
+      <c r="W189" t="str">
+        <v>1</v>
+      </c>
+      <c r="X189" t="str">
+        <v>5/17/26</v>
+      </c>
+      <c r="Y189" t="str">
+        <v>8/20/26</v>
+      </c>
+      <c r="Z189" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB189" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD189" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE189" t="str">
+        <v>Skipped: Intended practices disabled (program stage)</v>
+      </c>
+    </row>
+    <row r="190" xml:space="preserve">
+      <c r="A190" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B190" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C190" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D190" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E190" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F190" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J190" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K190" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L190" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M190" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N190" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O190" t="str">
+        <v>1</v>
+      </c>
+      <c r="P190" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q190" t="str">
+        <v>0</v>
+      </c>
+      <c r="R190" t="str">
+        <v>0</v>
+      </c>
+      <c r="S190" t="str">
+        <v>0</v>
+      </c>
+      <c r="T190" t="str">
+        <v>0</v>
+      </c>
+      <c r="U190" t="str">
+        <v>4</v>
+      </c>
+      <c r="V190" t="str">
+        <v>0</v>
+      </c>
+      <c r="W190" t="str">
+        <v>2</v>
+      </c>
+      <c r="X190" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y190" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z190" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB190" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD190" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE190" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="191" xml:space="preserve">
+      <c r="A191" t="str">
+        <v>(1252)</v>
+      </c>
+      <c r="B191" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group - HTX An Hoà</v>
+      </c>
+      <c r="C191" t="str">
+        <v>74110</v>
+      </c>
+      <c r="D191" t="str">
+        <v>946756347</v>
+      </c>
+      <c r="E191" t="str">
+        <v>TRẦN VĂN KHÁNH</v>
+      </c>
+      <c r="F191" t="str">
+        <v>HỢP TÁC XÃ NÔNG NGHIỆP AN HÒA</v>
+      </c>
+      <c r="J191" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K191" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L191" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M191" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N191" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O191" t="str">
+        <v>0</v>
+      </c>
+      <c r="P191" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q191" t="str">
+        <v>0</v>
+      </c>
+      <c r="R191" t="str">
+        <v>0</v>
+      </c>
+      <c r="S191" t="str">
+        <v>0</v>
+      </c>
+      <c r="T191" t="str">
+        <v>0</v>
+      </c>
+      <c r="U191" t="str">
+        <v>2</v>
+      </c>
+      <c r="V191" t="str">
+        <v>0</v>
+      </c>
+      <c r="W191" t="str">
+        <v>1</v>
+      </c>
+      <c r="X191" t="str">
+        <v>5/17/26</v>
+      </c>
+      <c r="Y191" t="str">
+        <v>8/20/26</v>
+      </c>
+      <c r="Z191" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB191" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD191" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE191" t="str">
+        <v>Skipped: Intended practices disabled (program stage)</v>
+      </c>
+    </row>
+    <row r="192" xml:space="preserve">
+      <c r="A192" t="str">
+        <v>(1175)</v>
+      </c>
+      <c r="B192" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group-HTX Hoà Thuận</v>
+      </c>
+      <c r="C192" t="str">
+        <v>73970</v>
+      </c>
+      <c r="D192" t="str">
+        <v>919813394</v>
+      </c>
+      <c r="E192" t="str">
+        <v>TRƯƠNG THỊ TIẾN</v>
+      </c>
+      <c r="F192" t="str">
+        <v>HỢP TÁC XÃ DỊCH VỤ TỔNG HỢP HÒA THUẬN</v>
+      </c>
+      <c r="J192" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K192" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L192" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="M192" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N192" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O192" t="str">
+        <v>1</v>
+      </c>
+      <c r="P192" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q192" t="str">
+        <v>0</v>
+      </c>
+      <c r="R192" t="str">
+        <v>0</v>
+      </c>
+      <c r="S192" t="str">
+        <v>0</v>
+      </c>
+      <c r="T192" t="str">
+        <v>0</v>
+      </c>
+      <c r="U192" t="str">
+        <v>4</v>
+      </c>
+      <c r="V192" t="str">
+        <v>0</v>
+      </c>
+      <c r="W192" t="str">
+        <v>2</v>
+      </c>
+      <c r="X192" t="str">
+        <v>4/20/26</v>
+      </c>
+      <c r="Y192" t="str">
+        <v>7/24/26</v>
+      </c>
+      <c r="Z192" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB192" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD192" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE192" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="193" xml:space="preserve">
+      <c r="A193" t="str">
+        <v>(1252)</v>
+      </c>
+      <c r="B193" t="str">
+        <v>(1) Viet Nga Group, (2) Việt Nga Group - HTX An Hoà</v>
+      </c>
+      <c r="C193" t="str">
+        <v>74110</v>
+      </c>
+      <c r="D193" t="str">
+        <v>946756347</v>
+      </c>
+      <c r="E193" t="str">
+        <v>TRẦN VĂN KHÁNH</v>
+      </c>
+      <c r="F193" t="str">
+        <v>HỢP TÁC XÃ NÔNG NGHIỆP AN HÒA</v>
+      </c>
+      <c r="J193" t="str" xml:space="preserve">
+        <v xml:space="preserve">✅ Residue removal // Thu gom rơm rạ_x000d_
+✅ Rate reduction // Giảm lượng phân bón_x000d_
+✅ Reduced planting density // Giảm mật độ trồng_x000d_
+✅ Irrigation Management // Quản lý tưới tiêu</v>
+      </c>
+      <c r="K193" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="L193" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="M193" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="N193" t="str">
+        <v>NO</v>
+      </c>
+      <c r="O193" t="str">
+        <v>0</v>
+      </c>
+      <c r="P193" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q193" t="str">
+        <v>0</v>
+      </c>
+      <c r="R193" t="str">
+        <v>0</v>
+      </c>
+      <c r="S193" t="str">
+        <v>0</v>
+      </c>
+      <c r="T193" t="str">
+        <v>0</v>
+      </c>
+      <c r="U193" t="str">
+        <v>2</v>
+      </c>
+      <c r="V193" t="str">
+        <v>0</v>
+      </c>
+      <c r="W193" t="str">
+        <v>1</v>
+      </c>
+      <c r="X193" t="str">
+        <v>5/17/26</v>
+      </c>
+      <c r="Y193" t="str">
+        <v>8/20/26</v>
+      </c>
+      <c r="Z193" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="AB193" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="AD193" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AE193" t="str">
+        <v>Skipped: Intended practices disabled (program stage)</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE177"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE193"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor & getting by phone number
</commit_message>
<xml_diff>
--- a/cypress/fixtures/run-log.xlsx
+++ b/cypress/fixtures/run-log.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE603"/>
+  <dimension ref="A1:AE610"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str" xml:space="preserve">
@@ -49801,9 +49801,563 @@
         <v/>
       </c>
     </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>(2083)</v>
+      </c>
+      <c r="B604" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - NN số 2</v>
+      </c>
+      <c r="C604" t="str">
+        <v>65868</v>
+      </c>
+      <c r="D604" t="str">
+        <v>346700178</v>
+      </c>
+      <c r="E604" t="str">
+        <v>VÕ THỊ MẠNH</v>
+      </c>
+      <c r="F604" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G604" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H604" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="I604" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J604" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K604" t="str">
+        <v>1</v>
+      </c>
+      <c r="L604" t="str">
+        <v>0</v>
+      </c>
+      <c r="M604" t="str">
+        <v>0</v>
+      </c>
+      <c r="N604" t="str">
+        <v>0</v>
+      </c>
+      <c r="O604" t="str">
+        <v>0</v>
+      </c>
+      <c r="P604" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q604" t="str">
+        <v>3</v>
+      </c>
+      <c r="R604" t="str">
+        <v>0</v>
+      </c>
+      <c r="S604" t="str">
+        <v>2</v>
+      </c>
+      <c r="T604" t="str">
+        <v>4/28/26</v>
+      </c>
+      <c r="U604" t="str">
+        <v>8/1/26</v>
+      </c>
+      <c r="V604" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="W604" t="str">
+        <v>NGÂN</v>
+      </c>
+      <c r="X604" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z604" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA604" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>(2086)</v>
+      </c>
+      <c r="B605" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - NN số 2</v>
+      </c>
+      <c r="C605" t="str">
+        <v>65871</v>
+      </c>
+      <c r="D605" t="str">
+        <v>326167990</v>
+      </c>
+      <c r="E605" t="str">
+        <v>LÊ THỊ OANH</v>
+      </c>
+      <c r="F605" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G605" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H605" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="I605" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J605" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K605" t="str">
+        <v>1</v>
+      </c>
+      <c r="L605" t="str">
+        <v>0</v>
+      </c>
+      <c r="M605" t="str">
+        <v>0</v>
+      </c>
+      <c r="N605" t="str">
+        <v>0</v>
+      </c>
+      <c r="O605" t="str">
+        <v>0</v>
+      </c>
+      <c r="P605" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q605" t="str">
+        <v>3</v>
+      </c>
+      <c r="R605" t="str">
+        <v>0</v>
+      </c>
+      <c r="S605" t="str">
+        <v>2</v>
+      </c>
+      <c r="T605" t="str">
+        <v>4/28/26</v>
+      </c>
+      <c r="U605" t="str">
+        <v>8/1/26</v>
+      </c>
+      <c r="V605" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="W605" t="str">
+        <v>NGÂN</v>
+      </c>
+      <c r="X605" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z605" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA605" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>(2088)</v>
+      </c>
+      <c r="B606" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - NN số 2</v>
+      </c>
+      <c r="C606" t="str">
+        <v>65873</v>
+      </c>
+      <c r="D606" t="str">
+        <v>333342462</v>
+      </c>
+      <c r="E606" t="str">
+        <v>LÊ TẤN TÀI</v>
+      </c>
+      <c r="F606" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G606" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H606" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="I606" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J606" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K606" t="str">
+        <v>0</v>
+      </c>
+      <c r="L606" t="str">
+        <v>0</v>
+      </c>
+      <c r="M606" t="str">
+        <v>0</v>
+      </c>
+      <c r="N606" t="str">
+        <v>0</v>
+      </c>
+      <c r="O606" t="str">
+        <v>0</v>
+      </c>
+      <c r="P606" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q606" t="str">
+        <v>2</v>
+      </c>
+      <c r="R606" t="str">
+        <v>0</v>
+      </c>
+      <c r="S606" t="str">
+        <v>1</v>
+      </c>
+      <c r="T606" t="str">
+        <v>4/28/26</v>
+      </c>
+      <c r="U606" t="str">
+        <v>8/1/26</v>
+      </c>
+      <c r="V606" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="W606" t="str">
+        <v>NGÂN</v>
+      </c>
+      <c r="X606" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z606" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA606" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="str">
+        <v>(2108)</v>
+      </c>
+      <c r="B607" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - NN số 2</v>
+      </c>
+      <c r="C607" t="str">
+        <v>65922</v>
+      </c>
+      <c r="D607" t="str">
+        <v>354342105</v>
+      </c>
+      <c r="E607" t="str">
+        <v>GIANG VĂN HỌT</v>
+      </c>
+      <c r="F607" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G607" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H607" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="I607" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J607" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K607" t="str">
+        <v>0</v>
+      </c>
+      <c r="L607" t="str">
+        <v>0</v>
+      </c>
+      <c r="M607" t="str">
+        <v>0</v>
+      </c>
+      <c r="N607" t="str">
+        <v>0</v>
+      </c>
+      <c r="O607" t="str">
+        <v>0</v>
+      </c>
+      <c r="P607" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q607" t="str">
+        <v>4</v>
+      </c>
+      <c r="R607" t="str">
+        <v>0</v>
+      </c>
+      <c r="S607" t="str">
+        <v>3</v>
+      </c>
+      <c r="T607" t="str">
+        <v>4/28/26</v>
+      </c>
+      <c r="U607" t="str">
+        <v>8/1/26</v>
+      </c>
+      <c r="V607" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="W607" t="str">
+        <v>NGÂN</v>
+      </c>
+      <c r="X607" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z607" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA607" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="str">
+        <v>(2109)</v>
+      </c>
+      <c r="B608" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - NN số 2</v>
+      </c>
+      <c r="C608" t="str">
+        <v>65923</v>
+      </c>
+      <c r="D608" t="str">
+        <v>748939500</v>
+      </c>
+      <c r="E608" t="str">
+        <v>HỒ VĂN LONG</v>
+      </c>
+      <c r="F608" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G608" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H608" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="I608" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J608" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K608" t="str">
+        <v>0</v>
+      </c>
+      <c r="L608" t="str">
+        <v>0</v>
+      </c>
+      <c r="M608" t="str">
+        <v>0</v>
+      </c>
+      <c r="N608" t="str">
+        <v>0</v>
+      </c>
+      <c r="O608" t="str">
+        <v>0</v>
+      </c>
+      <c r="P608" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q608" t="str">
+        <v>4</v>
+      </c>
+      <c r="R608" t="str">
+        <v>0</v>
+      </c>
+      <c r="S608" t="str">
+        <v>3</v>
+      </c>
+      <c r="T608" t="str">
+        <v>4/28/26</v>
+      </c>
+      <c r="U608" t="str">
+        <v>8/1/26</v>
+      </c>
+      <c r="V608" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="W608" t="str">
+        <v>NGÂN</v>
+      </c>
+      <c r="X608" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z608" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA608" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="str">
+        <v>(3376)</v>
+      </c>
+      <c r="B609" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - HTX Tân Hà B</v>
+      </c>
+      <c r="C609" t="str">
+        <v>79855</v>
+      </c>
+      <c r="D609" t="str">
+        <v>974252489</v>
+      </c>
+      <c r="E609" t="str">
+        <v>TRƯƠNG THỊ TUYẾT NHUNG</v>
+      </c>
+      <c r="F609" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G609" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H609" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="I609" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J609" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K609" t="str">
+        <v>1</v>
+      </c>
+      <c r="L609" t="str">
+        <v>0</v>
+      </c>
+      <c r="M609" t="str">
+        <v>0</v>
+      </c>
+      <c r="N609" t="str">
+        <v>0</v>
+      </c>
+      <c r="O609" t="str">
+        <v>0</v>
+      </c>
+      <c r="P609" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q609" t="str">
+        <v>2</v>
+      </c>
+      <c r="R609" t="str">
+        <v>0</v>
+      </c>
+      <c r="S609" t="str">
+        <v>1</v>
+      </c>
+      <c r="T609" t="str">
+        <v>5/10/26</v>
+      </c>
+      <c r="U609" t="str">
+        <v>8/15/26</v>
+      </c>
+      <c r="V609" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="X609" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z609" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA609" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="str">
+        <v>(3376)</v>
+      </c>
+      <c r="B610" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - HTX Tân Hà B</v>
+      </c>
+      <c r="C610" t="str">
+        <v>79855</v>
+      </c>
+      <c r="D610" t="str">
+        <v>974252489</v>
+      </c>
+      <c r="E610" t="str">
+        <v>TRƯƠNG THỊ TUYẾT NHUNG</v>
+      </c>
+      <c r="F610" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G610" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H610" t="str">
+        <v>Female // Nữ</v>
+      </c>
+      <c r="I610" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J610" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K610" t="str">
+        <v>1</v>
+      </c>
+      <c r="L610" t="str">
+        <v>0</v>
+      </c>
+      <c r="M610" t="str">
+        <v>0</v>
+      </c>
+      <c r="N610" t="str">
+        <v>0</v>
+      </c>
+      <c r="O610" t="str">
+        <v>0</v>
+      </c>
+      <c r="P610" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q610" t="str">
+        <v>2</v>
+      </c>
+      <c r="R610" t="str">
+        <v>0</v>
+      </c>
+      <c r="S610" t="str">
+        <v>1</v>
+      </c>
+      <c r="T610" t="str">
+        <v>5/10/26</v>
+      </c>
+      <c r="U610" t="str">
+        <v>8/15/26</v>
+      </c>
+      <c r="V610" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="X610" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z610" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA610" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE603"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE610"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
enhance input timeout in tests
</commit_message>
<xml_diff>
--- a/cypress/fixtures/run-log.xlsx
+++ b/cypress/fixtures/run-log.xlsx
@@ -404,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE610"/>
+  <dimension ref="A1:AE611"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str" xml:space="preserve">
@@ -50355,9 +50355,86 @@
         <v/>
       </c>
     </row>
+    <row r="611">
+      <c r="A611" t="str">
+        <v>(1516)</v>
+      </c>
+      <c r="B611" t="str">
+        <v>(1) Viet Nga Group, (2) Viet Nga Group - HTX NN 285</v>
+      </c>
+      <c r="C611" t="str">
+        <v>80016</v>
+      </c>
+      <c r="D611" t="str">
+        <v>393822588</v>
+      </c>
+      <c r="E611" t="str">
+        <v>NGUYỄN NGỌC NAM</v>
+      </c>
+      <c r="F611" t="str">
+        <v>Intensive rice production // Trồng lúa thâm canh</v>
+      </c>
+      <c r="G611" t="str">
+        <v>Residue removal; Rate reduction; Reduced planting density; Irrigation Management;</v>
+      </c>
+      <c r="H611" t="str">
+        <v>Male // Nam</v>
+      </c>
+      <c r="I611" t="str">
+        <v>KINH</v>
+      </c>
+      <c r="J611" t="str">
+        <v>NO</v>
+      </c>
+      <c r="K611" t="str">
+        <v>0</v>
+      </c>
+      <c r="L611" t="str">
+        <v>0</v>
+      </c>
+      <c r="M611" t="str">
+        <v>0</v>
+      </c>
+      <c r="N611" t="str">
+        <v>0</v>
+      </c>
+      <c r="O611" t="str">
+        <v>0</v>
+      </c>
+      <c r="P611" t="str">
+        <v>0</v>
+      </c>
+      <c r="Q611" t="str">
+        <v>2</v>
+      </c>
+      <c r="R611" t="str">
+        <v>0</v>
+      </c>
+      <c r="S611" t="str">
+        <v>1</v>
+      </c>
+      <c r="T611" t="str">
+        <v>5/31/26</v>
+      </c>
+      <c r="U611" t="str">
+        <v>9/25/26</v>
+      </c>
+      <c r="V611" t="str">
+        <v>Có thể nhập MRV</v>
+      </c>
+      <c r="X611" t="str">
+        <v>Ngân</v>
+      </c>
+      <c r="Z611" t="str">
+        <v>Yes</v>
+      </c>
+      <c r="AA611" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AE610"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AE611"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>